<commit_message>
Update bitcoin_buys.xlsx after running on 2026-09-20
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1988,6 +1988,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>09/20/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>0.0009180199999999916</v>
+      </c>
+      <c r="C100" t="n">
+        <v>80880.59083680168</v>
+      </c>
+      <c r="D100" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-09-27
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2004,6 +2004,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>09/27/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>0.0008737700000000029</v>
+      </c>
+      <c r="C101" t="n">
+        <v>84976.59567162955</v>
+      </c>
+      <c r="D101" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-10-04
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2020,6 +2020,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>0.0005803199999999953</v>
+      </c>
+      <c r="C102" t="n">
+        <v>85297.76674938035</v>
+      </c>
+      <c r="D102" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-10-11
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2036,6 +2036,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>0.0005935700000000085</v>
+      </c>
+      <c r="C103" t="n">
+        <v>83393.70251191821</v>
+      </c>
+      <c r="D103" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-10-18
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2052,6 +2052,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10/18/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>0.0006034399999999968</v>
+      </c>
+      <c r="C104" t="n">
+        <v>82029.69640726545</v>
+      </c>
+      <c r="D104" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-10-25
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2068,6 +2068,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10/25/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>0.0006116899999999981</v>
+      </c>
+      <c r="C105" t="n">
+        <v>80923.34352368055</v>
+      </c>
+      <c r="D105" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>